<commit_message>
update to xsd schemas
</commit_message>
<xml_diff>
--- a/templates/oefen/oefen_bodem_template.xlsx
+++ b/templates/oefen/oefen_bodem_template.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12915" uniqueCount="2045">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12912" uniqueCount="2045">
   <si>
     <t>naam</t>
   </si>
@@ -6127,25 +6127,25 @@
     <t>Date generated</t>
   </si>
   <si>
-    <t>2026-02-10 16:32:13.449275</t>
+    <t>2026-03-31 16:51:46.791384</t>
   </si>
   <si>
     <t>version</t>
   </si>
   <si>
-    <t>2.2.3</t>
+    <t>2.3.0</t>
   </si>
   <si>
     <t>xdov-version</t>
   </si>
   <si>
-    <t>9.4.3</t>
+    <t>10.1.0</t>
   </si>
   <si>
     <t>schema-version</t>
   </si>
   <si>
-    <t>5.9.0</t>
+    <t>5.10.0</t>
   </si>
   <si>
     <t>mode</t>
@@ -47811,7 +47811,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:BH6"/>
+  <dimension ref="A1:BG6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="54.7109375" style="3" customWidth="1"/>
@@ -47871,10 +47871,9 @@
     <col min="57" max="57" width="34.7109375" style="3" customWidth="1"/>
     <col min="58" max="58" width="48.7109375" style="3" customWidth="1"/>
     <col min="59" max="59" width="40.7109375" customWidth="1"/>
-    <col min="60" max="60" width="10.7109375" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:60" hidden="1">
+    <row r="1" spans="1:59" hidden="1">
       <c r="A1" s="7" t="s">
         <v>1757</v>
       </c>
@@ -48052,11 +48051,8 @@
       <c r="BG1" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="BH1" s="1" t="s">
-        <v>1765</v>
-      </c>
-    </row>
-    <row r="2" spans="1:60" hidden="1">
+    </row>
+    <row r="2" spans="1:59" hidden="1">
       <c r="A2" s="8" t="s">
         <v>1758</v>
       </c>
@@ -48144,11 +48140,8 @@
       <c r="BE2" s="1"/>
       <c r="BF2" s="1"/>
       <c r="BG2" s="1"/>
-      <c r="BH2" s="1" t="s">
-        <v>1765</v>
-      </c>
-    </row>
-    <row r="3" spans="1:60" hidden="1">
+    </row>
+    <row r="3" spans="1:59" hidden="1">
       <c r="A3" s="8" t="s">
         <v>1758</v>
       </c>
@@ -48263,7 +48256,7 @@
       </c>
       <c r="BG3" s="1"/>
     </row>
-    <row r="4" spans="1:60" hidden="1">
+    <row r="4" spans="1:59" hidden="1">
       <c r="E4" s="8" t="s">
         <v>78</v>
       </c>
@@ -48346,7 +48339,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="5" spans="1:60" hidden="1">
+    <row r="5" spans="1:59" hidden="1">
       <c r="K5" s="8" t="s">
         <v>1774</v>
       </c>
@@ -48399,7 +48392,7 @@
         <v>1794</v>
       </c>
     </row>
-    <row r="6" spans="1:60">
+    <row r="6" spans="1:59">
       <c r="A6" s="7" t="s">
         <v>1757</v>
       </c>
@@ -48576,9 +48569,6 @@
       </c>
       <c r="BG6" s="1" t="s">
         <v>70</v>
-      </c>
-      <c r="BH6" s="1" t="s">
-        <v>1765</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added exception for monster xsd-schema
</commit_message>
<xml_diff>
--- a/templates/oefen/oefen_bodem_template.xlsx
+++ b/templates/oefen/oefen_bodem_template.xlsx
@@ -6133,19 +6133,19 @@
     <t>Date generated</t>
   </si>
   <si>
-    <t>2026-05-06 16:21:30.752882</t>
+    <t>2026-05-19 11:29:03.465817</t>
   </si>
   <si>
     <t>version</t>
   </si>
   <si>
-    <t>2.3.1</t>
+    <t>2.4.0</t>
   </si>
   <si>
     <t>xdov-version</t>
   </si>
   <si>
-    <t>10.1.0</t>
+    <t>10.2.0</t>
   </si>
   <si>
     <t>schema-version</t>

</xml_diff>

<commit_message>
Small bugfix to gml:posList
</commit_message>
<xml_diff>
--- a/templates/oefen/oefen_bodem_template.xlsx
+++ b/templates/oefen/oefen_bodem_template.xlsx
@@ -6133,13 +6133,13 @@
     <t>Date generated</t>
   </si>
   <si>
-    <t>2026-05-19 11:29:03.465817</t>
+    <t>2026-05-19 14:52:55.333274</t>
   </si>
   <si>
     <t>version</t>
   </si>
   <si>
-    <t>2.4.0</t>
+    <t>2.4.1</t>
   </si>
   <si>
     <t>xdov-version</t>

</xml_diff>